<commit_message>
Update param and import new vfx
</commit_message>
<xml_diff>
--- a/LubanConfig/DataTables/Datas/#ArtifactParam.xlsx
+++ b/LubanConfig/DataTables/Datas/#ArtifactParam.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Github\monster-ball\LubanConfig\DataTables\Datas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A45E50E6-447E-454C-9DB8-CD08A0BB8A14}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D0EDA055-20B1-43C6-8853-BD063FE19742}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -22,10 +22,36 @@
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
   <authors>
+    <author>Hannya T</author>
     <author/>
   </authors>
   <commentList>
-    <comment ref="C1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000001000000}">
+    <comment ref="B1" authorId="0" shapeId="0" xr:uid="{768C14FC-6E31-47AF-A906-3057EBFEC3E3}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Hannya T:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+Internal ID, can just follow the index format by making it i++
+</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="C1" authorId="1" shapeId="0" xr:uid="{00000000-0006-0000-0000-000001000000}">
       <text>
         <r>
           <rPr>
@@ -40,7 +66,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000002000000}">
+    <comment ref="D1" authorId="1" shapeId="0" xr:uid="{00000000-0006-0000-0000-000002000000}">
       <text>
         <r>
           <rPr>
@@ -50,12 +76,12 @@
             <scheme val="minor"/>
           </rPr>
           <t xml:space="preserve">String
-The displayed name for the artifact
+The displayed name for the artifact in artifact selection page
 </t>
         </r>
       </text>
     </comment>
-    <comment ref="E1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000003000000}">
+    <comment ref="E1" authorId="1" shapeId="0" xr:uid="{00000000-0006-0000-0000-000004000000}">
       <text>
         <r>
           <rPr>
@@ -64,13 +90,19 @@
             <rFont val="Arial"/>
             <scheme val="minor"/>
           </rPr>
-          <t>Int
-Purchase price of the artifact, in points</t>
+          <t xml:space="preserve">String
+Ball ID if the artifact is </t>
         </r>
-      </text>
-    </comment>
-    <comment ref="F1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000004000000}">
-      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <color rgb="FF000000"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+            <scheme val="minor"/>
+          </rPr>
+          <t xml:space="preserve">a </t>
+        </r>
         <r>
           <rPr>
             <sz val="10"/>
@@ -78,12 +110,11 @@
             <rFont val="Arial"/>
             <scheme val="minor"/>
           </rPr>
-          <t>String
-Ball ID if the artifact is ball specific upgrade</t>
+          <t>ball specific upgrade</t>
         </r>
       </text>
     </comment>
-    <comment ref="G1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000005000000}">
+    <comment ref="F1" authorId="1" shapeId="0" xr:uid="{00000000-0006-0000-0000-000005000000}">
       <text>
         <r>
           <rPr>
@@ -97,7 +128,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="H1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000006000000}">
+    <comment ref="G1" authorId="1" shapeId="0" xr:uid="{00000000-0006-0000-0000-000006000000}">
       <text>
         <r>
           <rPr>
@@ -111,7 +142,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="J1" authorId="0" shapeId="0" xr:uid="{A2122591-74C1-4294-AD07-432D4CD2F7B4}">
+    <comment ref="I1" authorId="1" shapeId="0" xr:uid="{A2122591-74C1-4294-AD07-432D4CD2F7B4}">
       <text>
         <r>
           <rPr>
@@ -125,7 +156,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="L1" authorId="0" shapeId="0" xr:uid="{A90D4D9A-BBFE-4379-8D00-4A158030AE29}">
+    <comment ref="K1" authorId="1" shapeId="0" xr:uid="{A90D4D9A-BBFE-4379-8D00-4A158030AE29}">
       <text>
         <r>
           <rPr>
@@ -139,7 +170,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="N1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000007000000}">
+    <comment ref="M1" authorId="1" shapeId="0" xr:uid="{00000000-0006-0000-0000-000007000000}">
       <text>
         <r>
           <rPr>
@@ -158,7 +189,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="38">
   <si>
     <t>##var</t>
   </si>
@@ -167,9 +198,6 @@
   </si>
   <si>
     <t>ArtifactName</t>
-  </si>
-  <si>
-    <t>ArtifactPrice</t>
   </si>
   <si>
     <t>BallRelation</t>
@@ -185,9 +213,6 @@
   </si>
   <si>
     <t>string</t>
-  </si>
-  <si>
-    <t>int</t>
   </si>
   <si>
     <t>#group</t>
@@ -305,7 +330,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -338,6 +363,19 @@
       <name val="Arial"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -596,8 +634,9 @@
   <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="4" max="4" width="17.33203125" customWidth="1"/>
-    <col min="5" max="6" width="18.6640625" customWidth="1"/>
-    <col min="7" max="7" width="50" customWidth="1"/>
+    <col min="5" max="5" width="18.6640625" customWidth="1"/>
+    <col min="6" max="6" width="71.88671875" customWidth="1"/>
+    <col min="7" max="7" width="20.109375" customWidth="1"/>
     <col min="8" max="8" width="15.21875" customWidth="1"/>
     <col min="10" max="10" width="14.33203125" customWidth="1"/>
   </cols>
@@ -607,7 +646,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>1</v>
@@ -621,29 +660,26 @@
       <c r="F1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="G1" s="1" t="s">
-        <v>5</v>
+      <c r="G1" s="2" t="s">
+        <v>14</v>
       </c>
       <c r="H1" s="2" t="s">
         <v>16</v>
       </c>
       <c r="I1" s="2" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="J1" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="K1" s="2" t="s">
+      <c r="L1" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="L1" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="M1" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="N1" s="1" t="s">
-        <v>6</v>
+      <c r="M1" s="1" t="s">
+        <v>5</v>
       </c>
       <c r="O1" s="1"/>
       <c r="P1" s="1"/>
@@ -663,46 +699,43 @@
     </row>
     <row r="2" spans="1:29" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="C2" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="B2" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>8</v>
-      </c>
       <c r="D2" s="1" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
-      <c r="G2" s="1" t="s">
-        <v>8</v>
+      <c r="G2" s="2" t="s">
+        <v>15</v>
       </c>
-      <c r="H2" s="2" t="s">
+      <c r="H2" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="I2" s="3" t="s">
-        <v>19</v>
+      <c r="I2" s="2" t="s">
+        <v>15</v>
       </c>
-      <c r="J2" s="2" t="s">
+      <c r="J2" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="K2" s="3" t="s">
-        <v>19</v>
+      <c r="K2" s="2" t="s">
+        <v>15</v>
       </c>
-      <c r="L2" s="2" t="s">
+      <c r="L2" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="M2" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="N2" s="2" t="s">
-        <v>17</v>
+      <c r="M2" s="2" t="s">
+        <v>15</v>
       </c>
       <c r="O2" s="1"/>
       <c r="P2" s="1"/>
@@ -722,7 +755,7 @@
     </row>
     <row r="3" spans="1:29" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B3" s="1"/>
       <c r="C3" s="1"/>
@@ -736,7 +769,6 @@
       <c r="K3" s="1"/>
       <c r="L3" s="1"/>
       <c r="M3" s="1"/>
-      <c r="N3" s="1"/>
       <c r="O3" s="1"/>
       <c r="P3" s="1"/>
       <c r="Q3" s="1"/>
@@ -755,7 +787,7 @@
     </row>
     <row r="4" spans="1:29" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="B4" s="1"/>
       <c r="C4" s="1"/>
@@ -769,7 +801,6 @@
       <c r="K4" s="1"/>
       <c r="L4" s="1"/>
       <c r="M4" s="1"/>
-      <c r="N4" s="1"/>
       <c r="O4" s="1"/>
       <c r="P4" s="1"/>
       <c r="Q4" s="1"/>
@@ -792,32 +823,29 @@
         <v>0</v>
       </c>
       <c r="C5" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="E5" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="D5" s="1" t="s">
+      <c r="F5" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="E5" s="1">
-        <v>100000</v>
+      <c r="G5" s="2" t="s">
+        <v>18</v>
       </c>
-      <c r="F5" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="G5" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="H5" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="I5" s="1">
+      <c r="H5" s="1">
         <v>4</v>
       </c>
+      <c r="I5" s="1"/>
       <c r="J5" s="1"/>
       <c r="K5" s="1"/>
       <c r="L5" s="1"/>
-      <c r="M5" s="1"/>
-      <c r="N5" s="2" t="s">
-        <v>26</v>
+      <c r="M5" s="2" t="s">
+        <v>24</v>
       </c>
       <c r="O5" s="1"/>
       <c r="P5" s="1"/>
@@ -841,30 +869,27 @@
         <v>1</v>
       </c>
       <c r="C6" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="E6" s="1"/>
+      <c r="F6" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="G6" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="D6" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="E6" s="1">
-        <v>50000</v>
-      </c>
-      <c r="F6" s="1"/>
-      <c r="G6" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="H6" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="I6" s="1">
+      <c r="H6" s="1">
         <v>200</v>
       </c>
+      <c r="I6" s="1"/>
       <c r="J6" s="1"/>
       <c r="K6" s="1"/>
       <c r="L6" s="1"/>
-      <c r="M6" s="1"/>
-      <c r="N6" s="2" t="s">
-        <v>27</v>
+      <c r="M6" s="2" t="s">
+        <v>25</v>
       </c>
       <c r="O6" s="1"/>
       <c r="P6" s="1"/>
@@ -888,34 +913,31 @@
         <v>2</v>
       </c>
       <c r="C7" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="E7" s="1"/>
+      <c r="F7" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="G7" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="D7" s="2" t="s">
+      <c r="H7" s="1">
+        <v>50</v>
+      </c>
+      <c r="I7" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="J7" s="1">
         <v>30</v>
       </c>
-      <c r="E7" s="1">
-        <v>75000</v>
-      </c>
-      <c r="F7" s="1"/>
-      <c r="G7" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="H7" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="I7" s="1">
-        <v>50</v>
-      </c>
-      <c r="J7" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="K7" s="1">
-        <v>30</v>
-      </c>
+      <c r="K7" s="1"/>
       <c r="L7" s="1"/>
-      <c r="M7" s="1"/>
-      <c r="N7" s="2" t="s">
-        <v>30</v>
+      <c r="M7" s="2" t="s">
+        <v>28</v>
       </c>
       <c r="O7" s="1"/>
       <c r="P7" s="1"/>
@@ -939,30 +961,27 @@
         <v>3</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
-      <c r="E8" s="1">
-        <v>40000</v>
-      </c>
-      <c r="F8" s="1"/>
-      <c r="G8" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="H8" s="2" t="s">
+      <c r="E8" s="1"/>
+      <c r="F8" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="I8" s="1">
+      <c r="G8" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="H8" s="1">
         <v>100</v>
       </c>
+      <c r="I8" s="1"/>
       <c r="J8" s="1"/>
       <c r="K8" s="1"/>
       <c r="L8" s="1"/>
-      <c r="M8" s="1"/>
-      <c r="N8" s="1" t="s">
-        <v>34</v>
+      <c r="M8" s="1" t="s">
+        <v>32</v>
       </c>
       <c r="O8" s="1"/>
       <c r="P8" s="1"/>
@@ -986,32 +1005,29 @@
         <v>4</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
-      <c r="E9" s="1">
-        <v>100000</v>
+      <c r="E9" s="2" t="s">
+        <v>35</v>
       </c>
       <c r="F9" s="2" t="s">
         <v>37</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
-      <c r="H9" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="I9" s="1">
+      <c r="H9" s="1">
         <v>30</v>
       </c>
+      <c r="I9" s="1"/>
       <c r="J9" s="1"/>
       <c r="K9" s="1"/>
       <c r="L9" s="1"/>
-      <c r="M9" s="1"/>
-      <c r="N9" s="1" t="s">
-        <v>36</v>
+      <c r="M9" s="1" t="s">
+        <v>34</v>
       </c>
       <c r="O9" s="1"/>
       <c r="P9" s="1"/>
@@ -1043,7 +1059,6 @@
       <c r="K10" s="1"/>
       <c r="L10" s="1"/>
       <c r="M10" s="1"/>
-      <c r="N10" s="1"/>
       <c r="O10" s="1"/>
       <c r="P10" s="1"/>
       <c r="Q10" s="1"/>

</xml_diff>

<commit_message>
Change artifact id data type
</commit_message>
<xml_diff>
--- a/LubanConfig/DataTables/Datas/#ArtifactParam.xlsx
+++ b/LubanConfig/DataTables/Datas/#ArtifactParam.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\601\monster-ball\LubanConfig\DataTables\Datas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ADB73DEB-06D6-4CB6-AABA-0C4D36B99329}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6A7D1785-4DBF-484B-9B9A-508140F72185}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="38280" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -59,6 +59,7 @@
             <sz val="10"/>
             <color rgb="FF000000"/>
             <rFont val="Arial"/>
+            <family val="2"/>
             <scheme val="minor"/>
           </rPr>
           <t xml:space="preserve">String
@@ -74,6 +75,7 @@
             <sz val="10"/>
             <color rgb="FF000000"/>
             <rFont val="Arial"/>
+            <family val="2"/>
             <scheme val="minor"/>
           </rPr>
           <t xml:space="preserve">String
@@ -89,6 +91,7 @@
             <sz val="10"/>
             <color rgb="FF000000"/>
             <rFont val="Arial"/>
+            <family val="2"/>
             <scheme val="minor"/>
           </rPr>
           <t xml:space="preserve">String
@@ -109,6 +112,7 @@
             <sz val="10"/>
             <color rgb="FF000000"/>
             <rFont val="Arial"/>
+            <family val="2"/>
             <scheme val="minor"/>
           </rPr>
           <t>ball specific upgrade</t>
@@ -122,6 +126,7 @@
             <sz val="10"/>
             <color rgb="FF000000"/>
             <rFont val="Arial"/>
+            <family val="2"/>
             <scheme val="minor"/>
           </rPr>
           <t>String
@@ -136,6 +141,7 @@
             <sz val="10"/>
             <color rgb="FF000000"/>
             <rFont val="Arial"/>
+            <family val="2"/>
             <scheme val="minor"/>
           </rPr>
           <t>[string, int]
@@ -150,6 +156,7 @@
             <sz val="10"/>
             <color rgb="FF000000"/>
             <rFont val="Arial"/>
+            <family val="2"/>
             <scheme val="minor"/>
           </rPr>
           <t>[string, int]
@@ -164,6 +171,7 @@
             <sz val="10"/>
             <color rgb="FF000000"/>
             <rFont val="Arial"/>
+            <family val="2"/>
             <scheme val="minor"/>
           </rPr>
           <t>[string, int]
@@ -178,6 +186,7 @@
             <sz val="10"/>
             <color rgb="FF000000"/>
             <rFont val="Arial"/>
+            <family val="2"/>
             <scheme val="minor"/>
           </rPr>
           <t xml:space="preserve">Artifact's ingame Icon
@@ -238,9 +247,6 @@
   </si>
   <si>
     <t>ID</t>
-  </si>
-  <si>
-    <t>ArtifactName</t>
   </si>
   <si>
     <t>BallRelation</t>
@@ -352,12 +358,6 @@
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
-    <t>FireTrailDuration</t>
-  </si>
-  <si>
-    <t>FireTrailSize</t>
-  </si>
-  <si>
     <t>Increase the duration of the fire trail left by the fireball by 30%</t>
   </si>
   <si>
@@ -367,13 +367,7 @@
     <t>FireCoal</t>
   </si>
   <si>
-    <t>FireTrailUptime</t>
-  </si>
-  <si>
     <t>Increase fireball's firetrail uptime by 30% when triggered.</t>
-  </si>
-  <si>
-    <t>SplitCount</t>
   </si>
   <si>
     <t>Splitball</t>
@@ -383,9 +377,6 @@
   </si>
   <si>
     <t>BallAttack</t>
-  </si>
-  <si>
-    <t>SplitSize</t>
   </si>
   <si>
     <t>Increase splitball's size by 30%.</t>
@@ -403,16 +394,10 @@
     <t>Reduce stenball's speed by 30%.</t>
   </si>
   <si>
-    <t>IceSize</t>
-  </si>
-  <si>
     <t>Iceball</t>
   </si>
   <si>
     <t>Increase the size of the ice zone left by the iceball by 30%.</t>
-  </si>
-  <si>
-    <t>IceAtk</t>
   </si>
   <si>
     <t>Increase iceball's attack by 30%, but increase skill requirment by 50%.</t>
@@ -424,13 +409,7 @@
     <t>Increase lightningball's zapping detection zone size by 30%, but make lightningball 40% more expensive to purchase.</t>
   </si>
   <si>
-    <t>LightningFrequency</t>
-  </si>
-  <si>
     <t>Increase lightningball's zapping frequency by 40%, but reduce its attack by 50%.</t>
-  </si>
-  <si>
-    <t>LightingReq</t>
   </si>
   <si>
     <t>Reduce lightningball's skill requirement by 30%, but reduce its speed by 30%.</t>
@@ -543,6 +522,46 @@
     <t>StenSpeed</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
+  <si>
+    <t>Artifacts.ID</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>FireTrailDuration</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>ArtifactName</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>FireTrailSize</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>FireTrailUptime</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>SplitSize</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>IceSize</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>IceAtk</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>LightningFrequency</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>LightingReq</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
 </sst>
 </file>
 
@@ -559,6 +578,7 @@
       <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -886,40 +906,40 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>1</v>
       </c>
       <c r="D1" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="E1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="F1" s="1" t="s">
-        <v>4</v>
-      </c>
       <c r="G1" s="2" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="H1" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="I1" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="J1" s="2" t="s">
+      <c r="K1" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="K1" s="2" t="s">
+      <c r="L1" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="L1" s="2" t="s">
-        <v>18</v>
-      </c>
       <c r="M1" s="1" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="O1" s="1"/>
       <c r="P1" s="1"/>
@@ -939,43 +959,43 @@
     </row>
     <row r="2" spans="1:29" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="D2" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="B2" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>7</v>
-      </c>
       <c r="E2" s="1" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="H2" s="3" t="s">
-        <v>61</v>
+        <v>51</v>
       </c>
       <c r="I2" s="2" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="J2" s="3" t="s">
-        <v>61</v>
+        <v>51</v>
       </c>
       <c r="K2" s="2" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="L2" s="3" t="s">
-        <v>61</v>
+        <v>51</v>
       </c>
       <c r="M2" s="2" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="O2" s="1"/>
       <c r="P2" s="1"/>
@@ -995,7 +1015,7 @@
     </row>
     <row r="3" spans="1:29" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B3" s="1"/>
       <c r="C3" s="1"/>
@@ -1027,7 +1047,7 @@
     </row>
     <row r="4" spans="1:29" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B4" s="1"/>
       <c r="C4" s="1"/>
@@ -1063,19 +1083,19 @@
         <v>0</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>33</v>
+        <v>79</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>71</v>
+        <v>61</v>
       </c>
       <c r="H5" s="1">
         <v>1.3</v>
@@ -1085,7 +1105,7 @@
       <c r="K5" s="1"/>
       <c r="L5" s="1"/>
       <c r="M5" s="2" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="O5" s="1"/>
       <c r="P5" s="1"/>
@@ -1109,19 +1129,19 @@
         <v>1</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>34</v>
+        <v>81</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>72</v>
+        <v>62</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>73</v>
+        <v>63</v>
       </c>
       <c r="H6" s="5">
         <v>1.3</v>
@@ -1129,7 +1149,7 @@
       <c r="K6" s="1"/>
       <c r="L6" s="1"/>
       <c r="M6" s="2" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="O6" s="1"/>
       <c r="P6" s="1"/>
@@ -1153,19 +1173,19 @@
         <v>2</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>38</v>
+        <v>82</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>74</v>
+        <v>64</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>75</v>
+        <v>65</v>
       </c>
       <c r="H7" s="5">
         <v>1.3</v>
@@ -1194,25 +1214,25 @@
         <v>3</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>40</v>
+        <v>67</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>76</v>
+        <v>66</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>41</v>
+        <v>30</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>42</v>
+        <v>37</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>77</v>
+        <v>67</v>
       </c>
       <c r="H8" s="1">
         <v>1.5</v>
       </c>
       <c r="I8" s="1" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="J8" s="5">
         <v>0.7</v>
@@ -1241,19 +1261,19 @@
         <v>4</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>44</v>
+        <v>83</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>78</v>
+        <v>68</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>41</v>
+        <v>36</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>45</v>
+        <v>39</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>79</v>
+        <v>69</v>
       </c>
       <c r="H9" s="1">
         <v>1.3</v>
@@ -1282,19 +1302,19 @@
         <v>5</v>
       </c>
       <c r="C10" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="E10" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="D10" s="2" t="s">
-        <v>80</v>
-      </c>
-      <c r="E10" s="2" t="s">
-        <v>31</v>
-      </c>
       <c r="F10" s="2" t="s">
-        <v>46</v>
+        <v>40</v>
       </c>
       <c r="G10" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="H10" s="1">
         <v>0.7</v>
@@ -1304,7 +1324,7 @@
       <c r="K10" s="1"/>
       <c r="L10" s="1"/>
       <c r="M10" s="1" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="O10" s="1"/>
       <c r="P10" s="1"/>
@@ -1327,20 +1347,20 @@
       <c r="B11" s="1">
         <v>6</v>
       </c>
-      <c r="C11" s="2" t="s">
-        <v>87</v>
+      <c r="C11" s="1" t="s">
+        <v>77</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>81</v>
+        <v>71</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>49</v>
+        <v>43</v>
       </c>
       <c r="G11" s="1" t="s">
-        <v>48</v>
+        <v>42</v>
       </c>
       <c r="H11" s="1">
         <v>1.3</v>
@@ -1373,19 +1393,19 @@
         <v>7</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>50</v>
+        <v>84</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>82</v>
+        <v>72</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>51</v>
+        <v>44</v>
       </c>
       <c r="F12" s="1" t="s">
-        <v>52</v>
+        <v>45</v>
       </c>
       <c r="G12" s="2" t="s">
-        <v>62</v>
+        <v>52</v>
       </c>
       <c r="H12" s="1">
         <v>1.3</v>
@@ -1418,25 +1438,25 @@
         <v>8</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>53</v>
+        <v>85</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>83</v>
+        <v>73</v>
       </c>
       <c r="E13" s="1" t="s">
-        <v>51</v>
+        <v>44</v>
       </c>
       <c r="F13" s="1" t="s">
-        <v>54</v>
+        <v>46</v>
       </c>
       <c r="G13" s="2" t="s">
-        <v>68</v>
+        <v>58</v>
       </c>
       <c r="H13" s="1">
         <v>1.3</v>
       </c>
       <c r="I13" s="2" t="s">
-        <v>63</v>
+        <v>53</v>
       </c>
       <c r="J13" s="5">
         <v>1.5</v>
@@ -1463,26 +1483,26 @@
       <c r="B14" s="1">
         <v>9</v>
       </c>
-      <c r="C14" s="2" t="s">
-        <v>64</v>
+      <c r="C14" s="1" t="s">
+        <v>54</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>84</v>
+        <v>74</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>65</v>
+        <v>55</v>
       </c>
       <c r="F14" s="6" t="s">
-        <v>56</v>
+        <v>48</v>
       </c>
       <c r="G14" s="2" t="s">
-        <v>64</v>
+        <v>54</v>
       </c>
       <c r="H14" s="1">
         <v>1.3</v>
       </c>
       <c r="I14" s="2" t="s">
-        <v>66</v>
+        <v>56</v>
       </c>
       <c r="J14" s="5">
         <v>1.4</v>
@@ -1510,25 +1530,25 @@
         <v>10</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>57</v>
+        <v>86</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>85</v>
+        <v>75</v>
       </c>
       <c r="E15" s="1" t="s">
-        <v>55</v>
+        <v>47</v>
       </c>
       <c r="F15" s="6" t="s">
-        <v>58</v>
+        <v>49</v>
       </c>
       <c r="G15" s="2" t="s">
-        <v>67</v>
+        <v>57</v>
       </c>
       <c r="H15" s="1">
         <v>0.6</v>
       </c>
       <c r="I15" s="2" t="s">
-        <v>68</v>
+        <v>58</v>
       </c>
       <c r="J15" s="5">
         <v>0.5</v>
@@ -1556,25 +1576,25 @@
         <v>11</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>59</v>
+        <v>87</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>86</v>
+        <v>76</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>65</v>
+        <v>55</v>
       </c>
       <c r="F16" s="1" t="s">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="G16" s="2" t="s">
-        <v>63</v>
+        <v>53</v>
       </c>
       <c r="H16" s="1">
         <v>0.7</v>
       </c>
       <c r="I16" s="2" t="s">
-        <v>69</v>
+        <v>59</v>
       </c>
       <c r="J16" s="5">
         <v>0.7</v>
@@ -1601,17 +1621,29 @@
       <c r="B17" s="1">
         <v>12</v>
       </c>
-      <c r="C17" s="1"/>
-      <c r="D17" s="1"/>
+      <c r="C17" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="D17" s="2" t="s">
+        <v>20</v>
+      </c>
       <c r="E17" s="1"/>
-      <c r="F17" s="1"/>
-      <c r="G17" s="1"/>
-      <c r="H17" s="1"/>
+      <c r="F17" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="G17" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="H17" s="1">
+        <v>200</v>
+      </c>
       <c r="I17" s="1"/>
       <c r="J17" s="1"/>
       <c r="K17" s="1"/>
       <c r="L17" s="1"/>
-      <c r="M17" s="1"/>
+      <c r="M17" s="2" t="s">
+        <v>20</v>
+      </c>
       <c r="N17" s="1"/>
       <c r="O17" s="1"/>
       <c r="P17" s="1"/>
@@ -1635,27 +1667,31 @@
         <v>13</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="E18" s="1"/>
-      <c r="F18" s="2" t="s">
-        <v>22</v>
+      <c r="F18" s="4" t="s">
+        <v>24</v>
       </c>
       <c r="G18" s="2" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="H18" s="1">
-        <v>200</v>
+        <v>50</v>
       </c>
-      <c r="I18" s="1"/>
-      <c r="J18" s="1"/>
+      <c r="I18" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="J18" s="1">
+        <v>30</v>
+      </c>
       <c r="K18" s="1"/>
       <c r="L18" s="1"/>
       <c r="M18" s="2" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="N18" s="1"/>
       <c r="O18" s="1"/>
@@ -1679,32 +1715,28 @@
       <c r="B19" s="1">
         <v>14</v>
       </c>
-      <c r="C19" s="2" t="s">
-        <v>24</v>
+      <c r="C19" s="1" t="s">
+        <v>27</v>
       </c>
-      <c r="D19" s="2" t="s">
-        <v>24</v>
+      <c r="D19" s="1" t="s">
+        <v>27</v>
       </c>
       <c r="E19" s="1"/>
-      <c r="F19" s="4" t="s">
-        <v>25</v>
+      <c r="F19" s="2" t="s">
+        <v>28</v>
       </c>
       <c r="G19" s="2" t="s">
         <v>26</v>
       </c>
       <c r="H19" s="1">
-        <v>50</v>
+        <v>100</v>
       </c>
-      <c r="I19" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="J19" s="1">
-        <v>30</v>
-      </c>
+      <c r="I19" s="1"/>
+      <c r="J19" s="1"/>
       <c r="K19" s="1"/>
       <c r="L19" s="1"/>
-      <c r="M19" s="2" t="s">
-        <v>24</v>
+      <c r="M19" s="1" t="s">
+        <v>27</v>
       </c>
       <c r="N19" s="1"/>
       <c r="O19" s="1"/>
@@ -1725,32 +1757,7 @@
     </row>
     <row r="20" spans="1:29" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="1"/>
-      <c r="B20" s="1">
-        <v>15</v>
-      </c>
-      <c r="C20" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="D20" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="E20" s="1"/>
-      <c r="F20" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="G20" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="H20" s="1">
-        <v>100</v>
-      </c>
-      <c r="I20" s="1"/>
-      <c r="J20" s="1"/>
-      <c r="K20" s="1"/>
-      <c r="L20" s="1"/>
-      <c r="M20" s="1" t="s">
-        <v>28</v>
-      </c>
+      <c r="B20" s="1"/>
       <c r="N20" s="1"/>
       <c r="O20" s="1"/>
       <c r="P20" s="1"/>

</xml_diff>

<commit_message>
Add 10 new artifact entries with icons
</commit_message>
<xml_diff>
--- a/LubanConfig/DataTables/Datas/#ArtifactParam.xlsx
+++ b/LubanConfig/DataTables/Datas/#ArtifactParam.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Github\monster-ball\LubanConfig\DataTables\Datas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F7C2736F-42ED-444C-ADB1-E8D23982F7B7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{08D0D25D-1E47-46AF-8165-54A7570F7906}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -241,7 +241,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="121" uniqueCount="96">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="147" uniqueCount="120">
   <si>
     <t>##var</t>
   </si>
@@ -313,19 +313,11 @@
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
-    <t>Increase player's starting gold by {0}.</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
     <t>Gold</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
     <t>Headhunter</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>Increase damage dealt towards monster by {0}%, but receive {1}% less point from all sources.</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
@@ -338,10 +330,6 @@
   </si>
   <si>
     <t>Stargate</t>
-  </si>
-  <si>
-    <t>Increase points granted by using the teleporter by {0}%.</t>
-    <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
     <t>Splitball</t>
@@ -596,6 +584,110 @@
     <t>BottledThunder</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
+  <si>
+    <t>Increase damage dealt towards monster by 30%, but receive 15% reduced point from all sources.</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Increase player's starting gold by 200.</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>HadronCollider</t>
+  </si>
+  <si>
+    <t>Increase points granted by using the teleporter by 30%.</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Increase points granted by using the bumper by 45%.</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>WhirlingFate</t>
+  </si>
+  <si>
+    <t>SpinnerPoint</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>BumperPoint</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>TeleportPoint</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>MonsterDamage</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>StartingGold</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>SwitchPoint</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Increase points granted by using the drop switch by 25%.</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Increase points granted by using the spinner by 35%.</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>PreciseMissile</t>
+  </si>
+  <si>
+    <t>DamagerPoint</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Increase points granted by using the damagers by 10%.</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>BigGameHunter</t>
+  </si>
+  <si>
+    <t>Big Game Hunter</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Precise Missile</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Clanky Lever</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Whirling Fate</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Hadron Collider</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>ClankyLever</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>GoldIncrease</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Increase all monster's gold drop by 30%, but increase all ball prices by 10%.</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>GoldDrop</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
 </sst>
 </file>
 
@@ -691,7 +783,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -701,9 +793,6 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -716,6 +805,12 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -959,7 +1054,7 @@
         <v>1</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>2</v>
@@ -1012,7 +1107,7 @@
         <v>13</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="D2" s="1" t="s">
         <v>6</v>
@@ -1027,19 +1122,19 @@
         <v>11</v>
       </c>
       <c r="H2" s="3" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="I2" s="2" t="s">
         <v>11</v>
       </c>
       <c r="J2" s="3" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="K2" s="2" t="s">
         <v>11</v>
       </c>
       <c r="L2" s="3" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="M2" s="2" t="s">
         <v>11</v>
@@ -1130,19 +1225,19 @@
         <v>0</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="E5" s="1" t="s">
         <v>9</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="H5" s="1">
         <v>1.3</v>
@@ -1151,8 +1246,8 @@
       <c r="J5" s="1"/>
       <c r="K5" s="1"/>
       <c r="L5" s="1"/>
-      <c r="M5" s="7" t="s">
-        <v>86</v>
+      <c r="M5" s="6" t="s">
+        <v>83</v>
       </c>
       <c r="O5" s="1"/>
       <c r="P5" s="1"/>
@@ -1176,27 +1271,27 @@
         <v>1</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="E6" s="1" t="s">
         <v>9</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
-      <c r="H6" s="5">
+      <c r="H6" s="4">
         <v>1.3</v>
       </c>
       <c r="K6" s="1"/>
       <c r="L6" s="1"/>
-      <c r="M6" s="7" t="s">
-        <v>85</v>
+      <c r="M6" s="6" t="s">
+        <v>82</v>
       </c>
       <c r="O6" s="1"/>
       <c r="P6" s="1"/>
@@ -1220,27 +1315,27 @@
         <v>2</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="E7" s="1" t="s">
         <v>9</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
-      <c r="H7" s="5">
+      <c r="H7" s="4">
         <v>1.3</v>
       </c>
       <c r="K7" s="1"/>
       <c r="L7" s="1"/>
-      <c r="M7" s="7" t="s">
-        <v>87</v>
+      <c r="M7" s="6" t="s">
+        <v>84</v>
       </c>
       <c r="O7" s="1"/>
       <c r="P7" s="1"/>
@@ -1264,33 +1359,33 @@
         <v>3</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="H8" s="1">
         <v>1.5</v>
       </c>
       <c r="I8" s="1" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
-      <c r="J8" s="5">
+      <c r="J8" s="4">
         <v>0.7</v>
       </c>
       <c r="K8" s="1"/>
       <c r="L8" s="1"/>
-      <c r="M8" s="7" t="s">
-        <v>88</v>
+      <c r="M8" s="6" t="s">
+        <v>85</v>
       </c>
       <c r="O8" s="1"/>
       <c r="P8" s="1"/>
@@ -1314,27 +1409,27 @@
         <v>4</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="E9" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="F9" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="F9" s="1" t="s">
-        <v>36</v>
-      </c>
       <c r="G9" s="2" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="H9" s="1">
         <v>1.3</v>
       </c>
       <c r="K9" s="1"/>
       <c r="L9" s="1"/>
-      <c r="M9" s="7" t="s">
-        <v>94</v>
+      <c r="M9" s="6" t="s">
+        <v>91</v>
       </c>
       <c r="O9" s="1"/>
       <c r="P9" s="1"/>
@@ -1358,19 +1453,19 @@
         <v>5</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="F10" s="2" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="G10" s="2" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="H10" s="1">
         <v>0.7</v>
@@ -1379,8 +1474,8 @@
       <c r="J10" s="1"/>
       <c r="K10" s="1"/>
       <c r="L10" s="1"/>
-      <c r="M10" s="7" t="s">
-        <v>89</v>
+      <c r="M10" s="6" t="s">
+        <v>86</v>
       </c>
       <c r="O10" s="1"/>
       <c r="P10" s="1"/>
@@ -1404,19 +1499,19 @@
         <v>6</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="G11" s="1" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="H11" s="1">
         <v>1.3</v>
@@ -1425,8 +1520,8 @@
       <c r="J11" s="1"/>
       <c r="K11" s="1"/>
       <c r="L11" s="1"/>
-      <c r="M11" s="7" t="s">
-        <v>90</v>
+      <c r="M11" s="6" t="s">
+        <v>87</v>
       </c>
       <c r="N11" s="1"/>
       <c r="O11" s="1"/>
@@ -1451,19 +1546,19 @@
         <v>7</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="F12" s="1" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="G12" s="2" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="H12" s="1">
         <v>1.3</v>
@@ -1472,8 +1567,8 @@
       <c r="J12" s="1"/>
       <c r="K12" s="1"/>
       <c r="L12" s="1"/>
-      <c r="M12" s="7" t="s">
-        <v>91</v>
+      <c r="M12" s="6" t="s">
+        <v>88</v>
       </c>
       <c r="N12" s="1"/>
       <c r="O12" s="1"/>
@@ -1498,31 +1593,31 @@
         <v>8</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="E13" s="1" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="F13" s="1" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="G13" s="2" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="H13" s="1">
         <v>1.3</v>
       </c>
       <c r="I13" s="2" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
-      <c r="J13" s="5">
+      <c r="J13" s="4">
         <v>1.5</v>
       </c>
-      <c r="M13" s="8" t="s">
-        <v>70</v>
+      <c r="M13" s="7" t="s">
+        <v>67</v>
       </c>
       <c r="N13" s="1"/>
       <c r="O13" s="1"/>
@@ -1547,31 +1642,31 @@
         <v>9</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
-      <c r="F14" s="6" t="s">
-        <v>45</v>
+      <c r="F14" s="5" t="s">
+        <v>42</v>
       </c>
       <c r="G14" s="2" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="H14" s="1">
         <v>1.3</v>
       </c>
       <c r="I14" s="2" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
-      <c r="J14" s="5">
+      <c r="J14" s="4">
         <v>1.4</v>
       </c>
-      <c r="M14" s="7" t="s">
-        <v>92</v>
+      <c r="M14" s="6" t="s">
+        <v>89</v>
       </c>
       <c r="N14" s="1"/>
       <c r="O14" s="1"/>
@@ -1596,31 +1691,31 @@
         <v>10</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="E15" s="1" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
-      <c r="F15" s="6" t="s">
-        <v>46</v>
+      <c r="F15" s="5" t="s">
+        <v>43</v>
       </c>
       <c r="G15" s="2" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="H15" s="1">
         <v>0.6</v>
       </c>
       <c r="I15" s="2" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
-      <c r="J15" s="5">
+      <c r="J15" s="4">
         <v>0.5</v>
       </c>
-      <c r="M15" s="7" t="s">
-        <v>93</v>
+      <c r="M15" s="6" t="s">
+        <v>90</v>
       </c>
       <c r="N15" s="1"/>
       <c r="O15" s="1"/>
@@ -1645,31 +1740,31 @@
         <v>11</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="F16" s="1" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="G16" s="2" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="H16" s="1">
         <v>0.7</v>
       </c>
       <c r="I16" s="2" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
-      <c r="J16" s="5">
+      <c r="J16" s="4">
         <v>0.7</v>
       </c>
-      <c r="M16" s="7" t="s">
-        <v>95</v>
+      <c r="M16" s="6" t="s">
+        <v>92</v>
       </c>
       <c r="N16" s="1"/>
       <c r="O16" s="1"/>
@@ -1693,18 +1788,18 @@
       <c r="B17" s="1">
         <v>12</v>
       </c>
-      <c r="C17" s="2" t="s">
-        <v>19</v>
+      <c r="C17" s="1" t="s">
+        <v>103</v>
       </c>
       <c r="D17" s="2" t="s">
         <v>19</v>
       </c>
       <c r="E17" s="1"/>
-      <c r="F17" s="2" t="s">
-        <v>20</v>
+      <c r="F17" s="1" t="s">
+        <v>94</v>
       </c>
       <c r="G17" s="2" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="H17" s="1">
         <v>200</v>
@@ -1713,7 +1808,7 @@
       <c r="J17" s="1"/>
       <c r="K17" s="1"/>
       <c r="L17" s="1"/>
-      <c r="M17" s="8" t="s">
+      <c r="M17" s="7" t="s">
         <v>19</v>
       </c>
       <c r="N17" s="1"/>
@@ -1733,37 +1828,37 @@
       <c r="AB17" s="1"/>
       <c r="AC17" s="1"/>
     </row>
-    <row r="18" spans="1:29" ht="15.75" customHeight="1">
+    <row r="18" spans="1:29" ht="39.6" customHeight="1">
       <c r="A18" s="1"/>
       <c r="B18" s="1">
         <v>13</v>
       </c>
-      <c r="C18" s="2" t="s">
+      <c r="C18" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="D18" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="E18" s="1"/>
+      <c r="F18" s="5" t="s">
+        <v>93</v>
+      </c>
+      <c r="G18" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="D18" s="2" t="s">
-        <v>22</v>
+      <c r="H18" s="1">
+        <v>1.3</v>
       </c>
-      <c r="E18" s="1"/>
-      <c r="F18" s="4" t="s">
+      <c r="I18" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="G18" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="H18" s="1">
-        <v>50</v>
-      </c>
-      <c r="I18" s="2" t="s">
-        <v>25</v>
-      </c>
       <c r="J18" s="1">
-        <v>30</v>
+        <v>0.85</v>
       </c>
       <c r="K18" s="1"/>
       <c r="L18" s="1"/>
-      <c r="M18" s="8" t="s">
-        <v>22</v>
+      <c r="M18" s="7" t="s">
+        <v>21</v>
       </c>
       <c r="N18" s="1"/>
       <c r="O18" s="1"/>
@@ -1787,28 +1882,28 @@
       <c r="B19" s="1">
         <v>14</v>
       </c>
-      <c r="C19" s="1" t="s">
-        <v>26</v>
+      <c r="C19" s="8" t="s">
+        <v>101</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="E19" s="1"/>
-      <c r="F19" s="2" t="s">
-        <v>27</v>
+      <c r="F19" s="1" t="s">
+        <v>96</v>
       </c>
       <c r="G19" s="2" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="H19" s="1">
-        <v>100</v>
+        <v>1.3</v>
       </c>
       <c r="I19" s="1"/>
       <c r="J19" s="1"/>
       <c r="K19" s="1"/>
       <c r="L19" s="1"/>
-      <c r="M19" s="7" t="s">
-        <v>26</v>
+      <c r="M19" s="6" t="s">
+        <v>24</v>
       </c>
       <c r="N19" s="1"/>
       <c r="O19" s="1"/>
@@ -1829,7 +1924,27 @@
     </row>
     <row r="20" spans="1:29" ht="15.75" customHeight="1">
       <c r="A20" s="1"/>
-      <c r="B20" s="1"/>
+      <c r="B20" s="1">
+        <v>15</v>
+      </c>
+      <c r="C20" s="9" t="s">
+        <v>100</v>
+      </c>
+      <c r="D20" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="F20" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="G20" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="H20" s="1">
+        <v>1.45</v>
+      </c>
+      <c r="M20" s="4" t="s">
+        <v>95</v>
+      </c>
       <c r="N20" s="1"/>
       <c r="O20" s="1"/>
       <c r="P20" s="1"/>
@@ -1849,7 +1964,27 @@
     </row>
     <row r="21" spans="1:29" ht="15.75" customHeight="1">
       <c r="A21" s="1"/>
-      <c r="B21" s="1"/>
+      <c r="B21" s="1">
+        <v>16</v>
+      </c>
+      <c r="C21" s="9" t="s">
+        <v>99</v>
+      </c>
+      <c r="D21" s="3" t="s">
+        <v>114</v>
+      </c>
+      <c r="F21" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="G21" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="H21" s="1">
+        <v>1.35</v>
+      </c>
+      <c r="M21" s="4" t="s">
+        <v>98</v>
+      </c>
       <c r="N21" s="1"/>
       <c r="O21" s="1"/>
       <c r="P21" s="1"/>
@@ -1869,18 +2004,32 @@
     </row>
     <row r="22" spans="1:29" ht="15.75" customHeight="1">
       <c r="A22" s="1"/>
-      <c r="B22" s="1"/>
-      <c r="C22" s="1"/>
-      <c r="D22" s="1"/>
+      <c r="B22" s="1">
+        <v>17</v>
+      </c>
+      <c r="C22" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="D22" s="1" t="s">
+        <v>113</v>
+      </c>
       <c r="E22" s="1"/>
-      <c r="F22" s="1"/>
-      <c r="G22" s="1"/>
-      <c r="H22" s="1"/>
+      <c r="F22" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="G22" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="H22" s="1">
+        <v>1.25</v>
+      </c>
       <c r="I22" s="1"/>
       <c r="J22" s="1"/>
       <c r="K22" s="1"/>
       <c r="L22" s="1"/>
-      <c r="M22" s="1"/>
+      <c r="M22" s="1" t="s">
+        <v>116</v>
+      </c>
       <c r="N22" s="1"/>
       <c r="O22" s="1"/>
       <c r="P22" s="1"/>
@@ -1900,18 +2049,32 @@
     </row>
     <row r="23" spans="1:29" ht="15.75" customHeight="1">
       <c r="A23" s="1"/>
-      <c r="B23" s="1"/>
-      <c r="C23" s="1"/>
-      <c r="D23" s="1"/>
+      <c r="B23" s="1">
+        <v>18</v>
+      </c>
+      <c r="C23" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="D23" s="1" t="s">
+        <v>112</v>
+      </c>
       <c r="E23" s="1"/>
-      <c r="F23" s="1"/>
-      <c r="G23" s="1"/>
-      <c r="H23" s="1"/>
+      <c r="F23" s="1" t="s">
+        <v>109</v>
+      </c>
+      <c r="G23" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="H23" s="1">
+        <v>1.1000000000000001</v>
+      </c>
       <c r="I23" s="1"/>
       <c r="J23" s="1"/>
       <c r="K23" s="1"/>
       <c r="L23" s="1"/>
-      <c r="M23" s="1"/>
+      <c r="M23" s="1" t="s">
+        <v>107</v>
+      </c>
       <c r="N23" s="1"/>
       <c r="O23" s="1"/>
       <c r="P23" s="1"/>
@@ -1931,18 +2094,36 @@
     </row>
     <row r="24" spans="1:29" ht="15.75" customHeight="1">
       <c r="A24" s="1"/>
-      <c r="B24" s="1"/>
-      <c r="C24" s="1"/>
-      <c r="D24" s="1"/>
+      <c r="B24" s="1">
+        <v>19</v>
+      </c>
+      <c r="C24" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="D24" s="1" t="s">
+        <v>111</v>
+      </c>
       <c r="E24" s="1"/>
-      <c r="F24" s="1"/>
-      <c r="G24" s="1"/>
-      <c r="H24" s="1"/>
-      <c r="I24" s="1"/>
-      <c r="J24" s="1"/>
+      <c r="F24" s="1" t="s">
+        <v>118</v>
+      </c>
+      <c r="G24" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="H24" s="1">
+        <v>1.3</v>
+      </c>
+      <c r="I24" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="J24" s="1">
+        <v>1.1000000000000001</v>
+      </c>
       <c r="K24" s="1"/>
       <c r="L24" s="1"/>
-      <c r="M24" s="1"/>
+      <c r="M24" s="1" t="s">
+        <v>110</v>
+      </c>
       <c r="N24" s="1"/>
       <c r="O24" s="1"/>
       <c r="P24" s="1"/>

</xml_diff>

<commit_message>
Add 7 new artifacts
</commit_message>
<xml_diff>
--- a/LubanConfig/DataTables/Datas/#ArtifactParam.xlsx
+++ b/LubanConfig/DataTables/Datas/#ArtifactParam.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Github\monster-ball\LubanConfig\DataTables\Datas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{08D0D25D-1E47-46AF-8165-54A7570F7906}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6434687F-EEE3-4720-9462-FC233894840C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -241,7 +241,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="147" uniqueCount="120">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="185" uniqueCount="154">
   <si>
     <t>##var</t>
   </si>
@@ -688,6 +688,139 @@
     <t>GoldDrop</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
+  <si>
+    <t>CubelinsLens</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>AgileProfessor</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>AlienPizza</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>CthulusTentacle</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>EyeofBoundary</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>CorruptedDisc</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>HotelBroom</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Cubelin's Lens</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Agile Professor</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Alien's Pizza</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Cthulu's Tentacle</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Eye of Boundary</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Corrupted Disc</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Broom from a hotel</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Increase all ball's size by 20%, but increase their price by 10%.</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Increase all ball's speed by 50%, but receive 30% less points from all sources.</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Gain 150 additional gold everytime you enter the shop.</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Increase all ball's critical strike damage by 200%, but reduce 50% of their critical strike chance.</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>You now enters the realm of the dead.</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Everytime you gain gold, it would be randomly multiplied between 150% or 50% of its original value.</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Spawn 1 additional monster in all milestones.</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>MonsterSpawn</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>GoldChange</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>DeathZone</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>BallCritChange</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>ExtraGold</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>BallSpeed</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>BallSize</t>
+  </si>
+  <si>
+    <t>BallSizeChange</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>BallSpeedChange</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>BallCritDmg</t>
+  </si>
+  <si>
+    <t>BallCritChance</t>
+  </si>
+  <si>
+    <t>MonsterSpawnSCount</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>1.5-0.5</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
 </sst>
 </file>
 
@@ -2143,18 +2276,36 @@
     </row>
     <row r="25" spans="1:29" ht="15.75" customHeight="1">
       <c r="A25" s="1"/>
-      <c r="B25" s="1"/>
-      <c r="C25" s="1"/>
-      <c r="D25" s="1"/>
+      <c r="B25" s="1">
+        <v>20</v>
+      </c>
+      <c r="C25" s="1" t="s">
+        <v>148</v>
+      </c>
+      <c r="D25" s="1" t="s">
+        <v>127</v>
+      </c>
       <c r="E25" s="1"/>
-      <c r="F25" s="1"/>
-      <c r="G25" s="1"/>
-      <c r="H25" s="1"/>
-      <c r="I25" s="1"/>
-      <c r="J25" s="1"/>
+      <c r="F25" s="1" t="s">
+        <v>134</v>
+      </c>
+      <c r="G25" s="1" t="s">
+        <v>147</v>
+      </c>
+      <c r="H25" s="1">
+        <v>1.2</v>
+      </c>
+      <c r="I25" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="J25" s="1">
+        <v>1.1000000000000001</v>
+      </c>
       <c r="K25" s="1"/>
       <c r="L25" s="1"/>
-      <c r="M25" s="1"/>
+      <c r="M25" s="1" t="s">
+        <v>120</v>
+      </c>
       <c r="N25" s="1"/>
       <c r="O25" s="1"/>
       <c r="P25" s="1"/>
@@ -2174,18 +2325,36 @@
     </row>
     <row r="26" spans="1:29" ht="15.75" customHeight="1">
       <c r="A26" s="1"/>
-      <c r="B26" s="1"/>
-      <c r="C26" s="1"/>
-      <c r="D26" s="1"/>
+      <c r="B26" s="1">
+        <v>21</v>
+      </c>
+      <c r="C26" s="1" t="s">
+        <v>149</v>
+      </c>
+      <c r="D26" s="1" t="s">
+        <v>128</v>
+      </c>
       <c r="E26" s="1"/>
-      <c r="F26" s="1"/>
-      <c r="G26" s="1"/>
-      <c r="H26" s="1"/>
-      <c r="I26" s="1"/>
-      <c r="J26" s="1"/>
+      <c r="F26" s="1" t="s">
+        <v>135</v>
+      </c>
+      <c r="G26" s="1" t="s">
+        <v>146</v>
+      </c>
+      <c r="H26" s="1">
+        <v>1.5</v>
+      </c>
+      <c r="I26" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="J26" s="1">
+        <v>0.7</v>
+      </c>
       <c r="K26" s="1"/>
       <c r="L26" s="1"/>
-      <c r="M26" s="1"/>
+      <c r="M26" s="1" t="s">
+        <v>121</v>
+      </c>
       <c r="N26" s="1"/>
       <c r="O26" s="1"/>
       <c r="P26" s="1"/>
@@ -2205,18 +2374,32 @@
     </row>
     <row r="27" spans="1:29" ht="15.75" customHeight="1">
       <c r="A27" s="1"/>
-      <c r="B27" s="1"/>
-      <c r="C27" s="1"/>
-      <c r="D27" s="1"/>
+      <c r="B27" s="1">
+        <v>22</v>
+      </c>
+      <c r="C27" s="1" t="s">
+        <v>145</v>
+      </c>
+      <c r="D27" s="1" t="s">
+        <v>129</v>
+      </c>
       <c r="E27" s="1"/>
-      <c r="F27" s="1"/>
-      <c r="G27" s="1"/>
-      <c r="H27" s="1"/>
+      <c r="F27" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="G27" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="H27" s="1">
+        <v>150</v>
+      </c>
       <c r="I27" s="1"/>
       <c r="J27" s="1"/>
       <c r="K27" s="1"/>
       <c r="L27" s="1"/>
-      <c r="M27" s="1"/>
+      <c r="M27" s="1" t="s">
+        <v>122</v>
+      </c>
       <c r="N27" s="1"/>
       <c r="O27" s="1"/>
       <c r="P27" s="1"/>
@@ -2236,18 +2419,36 @@
     </row>
     <row r="28" spans="1:29" ht="15.75" customHeight="1">
       <c r="A28" s="1"/>
-      <c r="B28" s="1"/>
-      <c r="C28" s="1"/>
-      <c r="D28" s="1"/>
+      <c r="B28" s="1">
+        <v>23</v>
+      </c>
+      <c r="C28" s="1" t="s">
+        <v>144</v>
+      </c>
+      <c r="D28" s="1" t="s">
+        <v>130</v>
+      </c>
       <c r="E28" s="1"/>
-      <c r="F28" s="1"/>
-      <c r="G28" s="1"/>
-      <c r="H28" s="1"/>
-      <c r="I28" s="1"/>
-      <c r="J28" s="1"/>
+      <c r="F28" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="G28" s="1" t="s">
+        <v>150</v>
+      </c>
+      <c r="H28" s="1">
+        <v>2</v>
+      </c>
+      <c r="I28" s="1" t="s">
+        <v>151</v>
+      </c>
+      <c r="J28" s="1">
+        <v>0.5</v>
+      </c>
       <c r="K28" s="1"/>
       <c r="L28" s="1"/>
-      <c r="M28" s="1"/>
+      <c r="M28" s="1" t="s">
+        <v>123</v>
+      </c>
       <c r="N28" s="1"/>
       <c r="O28" s="1"/>
       <c r="P28" s="1"/>
@@ -2267,18 +2468,28 @@
     </row>
     <row r="29" spans="1:29" ht="15.75" customHeight="1">
       <c r="A29" s="1"/>
-      <c r="B29" s="1"/>
-      <c r="C29" s="1"/>
-      <c r="D29" s="1"/>
+      <c r="B29" s="1">
+        <v>24</v>
+      </c>
+      <c r="C29" s="1" t="s">
+        <v>143</v>
+      </c>
+      <c r="D29" s="1" t="s">
+        <v>131</v>
+      </c>
       <c r="E29" s="1"/>
-      <c r="F29" s="1"/>
+      <c r="F29" s="1" t="s">
+        <v>138</v>
+      </c>
       <c r="G29" s="1"/>
       <c r="H29" s="1"/>
       <c r="I29" s="1"/>
       <c r="J29" s="1"/>
       <c r="K29" s="1"/>
       <c r="L29" s="1"/>
-      <c r="M29" s="1"/>
+      <c r="M29" s="1" t="s">
+        <v>124</v>
+      </c>
       <c r="N29" s="1"/>
       <c r="O29" s="1"/>
       <c r="P29" s="1"/>
@@ -2298,18 +2509,32 @@
     </row>
     <row r="30" spans="1:29" ht="15.75" customHeight="1">
       <c r="A30" s="1"/>
-      <c r="B30" s="1"/>
-      <c r="C30" s="1"/>
-      <c r="D30" s="1"/>
+      <c r="B30" s="1">
+        <v>25</v>
+      </c>
+      <c r="C30" s="1" t="s">
+        <v>142</v>
+      </c>
+      <c r="D30" s="1" t="s">
+        <v>132</v>
+      </c>
       <c r="E30" s="1"/>
-      <c r="F30" s="1"/>
-      <c r="G30" s="1"/>
-      <c r="H30" s="1"/>
+      <c r="F30" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="G30" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="H30" s="1" t="s">
+        <v>153</v>
+      </c>
       <c r="I30" s="1"/>
       <c r="J30" s="1"/>
       <c r="K30" s="1"/>
       <c r="L30" s="1"/>
-      <c r="M30" s="1"/>
+      <c r="M30" s="1" t="s">
+        <v>125</v>
+      </c>
       <c r="N30" s="1"/>
       <c r="O30" s="1"/>
       <c r="P30" s="1"/>
@@ -2329,18 +2554,32 @@
     </row>
     <row r="31" spans="1:29" ht="15.75" customHeight="1">
       <c r="A31" s="1"/>
-      <c r="B31" s="1"/>
-      <c r="C31" s="1"/>
-      <c r="D31" s="1"/>
+      <c r="B31" s="1">
+        <v>26</v>
+      </c>
+      <c r="C31" s="1" t="s">
+        <v>141</v>
+      </c>
+      <c r="D31" s="1" t="s">
+        <v>133</v>
+      </c>
       <c r="E31" s="1"/>
-      <c r="F31" s="1"/>
-      <c r="G31" s="1"/>
-      <c r="H31" s="1"/>
+      <c r="F31" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="G31" s="1" t="s">
+        <v>152</v>
+      </c>
+      <c r="H31" s="1">
+        <v>1</v>
+      </c>
       <c r="I31" s="1"/>
       <c r="J31" s="1"/>
       <c r="K31" s="1"/>
       <c r="L31" s="1"/>
-      <c r="M31" s="1"/>
+      <c r="M31" s="1" t="s">
+        <v>126</v>
+      </c>
       <c r="N31" s="1"/>
       <c r="O31" s="1"/>
       <c r="P31" s="1"/>

</xml_diff>